<commit_message>
IMPORT-4 wip: import4-layers suite, ID match first, undo fixes
</commit_message>
<xml_diff>
--- a/tests/fixtures/import/event-guest-list-scrubbed.xlsx
+++ b/tests/fixtures/import/event-guest-list-scrubbed.xlsx
@@ -2029,10 +2029,7 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>null Treadwell</v>
-      </c>
-      <c r="B66" t="str">
-        <v>null.treadwell@example.net</v>
+        <v>Treadwell</v>
       </c>
       <c r="C66" t="str">
         <v>Yes</v>
@@ -3097,10 +3094,10 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>Theo Castilloe</v>
+        <v>Alma Arnolde</v>
       </c>
       <c r="B108" t="str">
-        <v>theo.castilloe0@example.net</v>
+        <v>alma.arnolde0@example.net</v>
       </c>
       <c r="C108" t="str">
         <v>Yes</v>
@@ -3123,10 +3120,10 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>Lucinda Jenningse</v>
+        <v>Theo Bennette</v>
       </c>
       <c r="B109" t="str">
-        <v>lucinda.jenningse1@example.net</v>
+        <v>theo.bennette1@example.net</v>
       </c>
       <c r="C109" t="str">
         <v>Yes</v>
@@ -3149,10 +3146,10 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>Felix Quinteroe</v>
+        <v>Priya Castilloe</v>
       </c>
       <c r="B110" t="str">
-        <v>felix.quinteroe2@example.net</v>
+        <v>priya.castilloe2@example.net</v>
       </c>
       <c r="C110" t="str">
         <v>Yes</v>
@@ -3175,10 +3172,10 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>Ines Arnolde</v>
+        <v>Jonah Dawsone</v>
       </c>
       <c r="B111" t="str">
-        <v>ines.arnolde3@example.net</v>
+        <v>jonah.dawsone3@example.net</v>
       </c>
       <c r="C111" t="str">
         <v>Yes</v>
@@ -3201,10 +3198,10 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>Elliot Hollowaye</v>
+        <v>Lucinda Ellisone</v>
       </c>
       <c r="B112" t="str">
-        <v>elliot.hollowaye4@example.net</v>
+        <v>lucinda.ellisone4@example.net</v>
       </c>
       <c r="C112" t="str">
         <v>Yes</v>
@@ -3227,10 +3224,10 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>Rosalind Okafore</v>
+        <v>Omar Fairbankse</v>
       </c>
       <c r="B113" t="str">
-        <v>rosalind.okafore5@example.net</v>
+        <v>omar.fairbankse5@example.net</v>
       </c>
       <c r="C113" t="str">
         <v>Yes</v>
@@ -3253,10 +3250,10 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>Barnaby Valdiviae</v>
+        <v>Beatrice Garnere</v>
       </c>
       <c r="B114" t="str">
-        <v>barnaby.valdiviae6@example.net</v>
+        <v>beatrice.garnere6@example.net</v>
       </c>
       <c r="C114" t="str">
         <v>Yes</v>
@@ -3279,10 +3276,10 @@
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>Marisol Fairbankse</v>
+        <v>Felix Hollowaye</v>
       </c>
       <c r="B115" t="str">
-        <v>marisol.fairbankse7@example.net</v>
+        <v>felix.hollowaye7@example.net</v>
       </c>
       <c r="C115" t="str">
         <v>Yes</v>
@@ -3305,10 +3302,10 @@
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>Priya Mercere</v>
+        <v>Harriet Ibarrae</v>
       </c>
       <c r="B116" t="str">
-        <v>priya.mercere8@example.net</v>
+        <v>harriet.ibarrae8@example.net</v>
       </c>
       <c r="C116" t="str">
         <v>Yes</v>
@@ -3331,10 +3328,10 @@
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>Omar Thackeraye</v>
+        <v>Marcus Jenningse</v>
       </c>
       <c r="B117" t="str">
-        <v>omar.thackeraye9@example.net</v>
+        <v>marcus.jenningse9@example.net</v>
       </c>
       <c r="C117" t="str">
         <v>Yes</v>
@@ -3357,10 +3354,10 @@
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>Harriet Dawsone</v>
+        <v>Ines Kowalskie</v>
       </c>
       <c r="B118" t="str">
-        <v>harriet.dawsone10@example.net</v>
+        <v>ines.kowalskie10@example.net</v>
       </c>
       <c r="C118" t="str">
         <v>Yes</v>
@@ -3383,10 +3380,10 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>Gordon Kowalskie</v>
+        <v>Gordon Langforde</v>
       </c>
       <c r="B119" t="str">
-        <v>gordon.kowalskie11@example.net</v>
+        <v>gordon.langforde11@example.net</v>
       </c>
       <c r="C119" t="str">
         <v>Yes</v>
@@ -3409,10 +3406,10 @@
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>Wren Rasmussene</v>
+        <v>Tamsin Mercere</v>
       </c>
       <c r="B120" t="str">
-        <v>wren.rasmussene12@example.net</v>
+        <v>tamsin.mercere12@example.net</v>
       </c>
       <c r="C120" t="str">
         <v>Yes</v>
@@ -3435,10 +3432,10 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>Caspian Bennette</v>
+        <v>Elliot Nakamurae</v>
       </c>
       <c r="B121" t="str">
-        <v>caspian.bennette13@example.net</v>
+        <v>elliot.nakamurae13@example.net</v>
       </c>
       <c r="C121" t="str">
         <v>Yes</v>
@@ -3461,10 +3458,10 @@
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>Leonie Ibarrae</v>
+        <v>Wren Okafore</v>
       </c>
       <c r="B122" t="str">
-        <v>leonie.ibarrae14@example.net</v>
+        <v>wren.okafore14@example.net</v>
       </c>
       <c r="C122" t="str">
         <v>Yes</v>
@@ -3487,10 +3484,10 @@
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>Alma Prescotte</v>
+        <v>Desmond Prescotte</v>
       </c>
       <c r="B123" t="str">
-        <v>alma.prescotte15@example.net</v>
+        <v>desmond.prescotte15@example.net</v>
       </c>
       <c r="C123" t="str">
         <v>Yes</v>
@@ -3513,10 +3510,10 @@
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>Jonah Whitlocke</v>
+        <v>Rosalind Quinteroe</v>
       </c>
       <c r="B124" t="str">
-        <v>jonah.whitlocke16@example.net</v>
+        <v>rosalind.quinteroe16@example.net</v>
       </c>
       <c r="C124" t="str">
         <v>Yes</v>
@@ -3539,10 +3536,10 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>Beatrice Garnere</v>
+        <v>Caspian Rasmussene</v>
       </c>
       <c r="B125" t="str">
-        <v>beatrice.garnere17@example.net</v>
+        <v>caspian.rasmussene17@example.net</v>
       </c>
       <c r="C125" t="str">
         <v>Yes</v>
@@ -3565,10 +3562,10 @@
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>Marcus Nakamurae</v>
+        <v>Odette Sorensene</v>
       </c>
       <c r="B126" t="str">
-        <v>marcus.nakamurae18@example.net</v>
+        <v>odette.sorensene18@example.net</v>
       </c>
       <c r="C126" t="str">
         <v>Yes</v>
@@ -3591,10 +3588,10 @@
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>Tamsin Underhille</v>
+        <v>Barnaby Thackeraye</v>
       </c>
       <c r="B127" t="str">
-        <v>tamsin.underhille19@example.net</v>
+        <v>barnaby.thackeraye19@example.net</v>
       </c>
       <c r="C127" t="str">
         <v>Yes</v>
@@ -3617,10 +3614,10 @@
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>Desmond Ellisone</v>
+        <v>Leonie Underhille</v>
       </c>
       <c r="B128" t="str">
-        <v>desmond.ellisone20@example.net</v>
+        <v>leonie.underhille20@example.net</v>
       </c>
       <c r="C128" t="str">
         <v>Yes</v>
@@ -3643,10 +3640,10 @@
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>Odette Langforde</v>
+        <v>Tobias Valdiviae</v>
       </c>
       <c r="B129" t="str">
-        <v>odette.langforde21@example.net</v>
+        <v>tobias.valdiviae21@example.net</v>
       </c>
       <c r="C129" t="str">
         <v>Yes</v>
@@ -3669,10 +3666,10 @@
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>Tobias Sorensene</v>
+        <v>Marisol Whitlocke</v>
       </c>
       <c r="B130" t="str">
-        <v>tobias.sorensene22@example.net</v>
+        <v>marisol.whitlocke22@example.net</v>
       </c>
       <c r="C130" t="str">
         <v>Yes</v>
@@ -3695,10 +3692,10 @@
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>Theo Castilloe</v>
+        <v>Alma Dawsone</v>
       </c>
       <c r="B131" t="str">
-        <v>theo.castilloe23@example.net</v>
+        <v>alma.dawsone23@example.net</v>
       </c>
       <c r="C131" t="str">
         <v>Yes</v>
@@ -3721,10 +3718,10 @@
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>Lucinda Jenningse</v>
+        <v>Theo Ellisone</v>
       </c>
       <c r="B132" t="str">
-        <v>lucinda.jenningse24@example.net</v>
+        <v>theo.ellisone24@example.net</v>
       </c>
       <c r="C132" t="str">
         <v>Yes</v>
@@ -3747,10 +3744,10 @@
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>Felix Quinteroe</v>
+        <v>Priya Fairbankse</v>
       </c>
       <c r="B133" t="str">
-        <v>felix.quinteroe25@example.net</v>
+        <v>priya.fairbankse25@example.net</v>
       </c>
       <c r="C133" t="str">
         <v>Yes</v>
@@ -3773,10 +3770,10 @@
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>Ines Arnolde</v>
+        <v>Jonah Garnere</v>
       </c>
       <c r="B134" t="str">
-        <v>ines.arnolde26@example.net</v>
+        <v>jonah.garnere26@example.net</v>
       </c>
       <c r="C134" t="str">
         <v>Yes</v>
@@ -3799,10 +3796,10 @@
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>Elliot Hollowaye</v>
+        <v>Lucinda Hollowaye</v>
       </c>
       <c r="B135" t="str">
-        <v>elliot.hollowaye27@example.net</v>
+        <v>lucinda.hollowaye27@example.net</v>
       </c>
       <c r="C135" t="str">
         <v>Yes</v>
@@ -3825,10 +3822,10 @@
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>Rosalind Okafore</v>
+        <v>Omar Ibarrae</v>
       </c>
       <c r="B136" t="str">
-        <v>rosalind.okafore28@example.net</v>
+        <v>omar.ibarrae28@example.net</v>
       </c>
       <c r="C136" t="str">
         <v>Yes</v>
@@ -3851,10 +3848,10 @@
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>Barnaby Valdiviae</v>
+        <v>Beatrice Jenningse</v>
       </c>
       <c r="B137" t="str">
-        <v>barnaby.valdiviae29@example.net</v>
+        <v>beatrice.jenningse29@example.net</v>
       </c>
       <c r="C137" t="str">
         <v>Yes</v>
@@ -3877,10 +3874,10 @@
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>Marisol Fairbankse</v>
+        <v>Felix Kowalskie</v>
       </c>
       <c r="B138" t="str">
-        <v>marisol.fairbankse30@example.net</v>
+        <v>felix.kowalskie30@example.net</v>
       </c>
       <c r="C138" t="str">
         <v>Yes</v>
@@ -3894,10 +3891,10 @@
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>Priya Mercere</v>
+        <v>Harriet Langforde</v>
       </c>
       <c r="B139" t="str">
-        <v>priya.mercere31@example.net</v>
+        <v>harriet.langforde31@example.net</v>
       </c>
       <c r="C139" t="str">
         <v>Yes</v>
@@ -3911,10 +3908,10 @@
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>Omar Thackeraye</v>
+        <v>Marcus Mercere</v>
       </c>
       <c r="B140" t="str">
-        <v>omar.thackeraye32@example.net</v>
+        <v>marcus.mercere32@example.net</v>
       </c>
       <c r="C140" t="str">
         <v>Yes</v>
@@ -3928,10 +3925,10 @@
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>Harriet Dawsone</v>
+        <v>Ines Nakamurae</v>
       </c>
       <c r="B141" t="str">
-        <v>harriet.dawsone33@example.net</v>
+        <v>ines.nakamurae33@example.net</v>
       </c>
       <c r="C141" t="str">
         <v>Yes</v>
@@ -3945,10 +3942,10 @@
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>Gordon Kowalskie</v>
+        <v>Gordon Okafore</v>
       </c>
       <c r="B142" t="str">
-        <v>gordon.kowalskie34@example.net</v>
+        <v>gordon.okafore34@example.net</v>
       </c>
       <c r="C142" t="str">
         <v>Yes</v>
@@ -3962,10 +3959,10 @@
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>Wren Rasmussene</v>
+        <v>Tamsin Prescotte</v>
       </c>
       <c r="B143" t="str">
-        <v>wren.rasmussene35@example.net</v>
+        <v>tamsin.prescotte35@example.net</v>
       </c>
       <c r="C143" t="str">
         <v>Yes</v>
@@ -3979,10 +3976,10 @@
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>Caspian Bennette</v>
+        <v>Elliot Quinteroe</v>
       </c>
       <c r="B144" t="str">
-        <v>caspian.bennette36@example.net</v>
+        <v>elliot.quinteroe36@example.net</v>
       </c>
       <c r="C144" t="str">
         <v>Yes</v>
@@ -3996,10 +3993,10 @@
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>Leonie Ibarrae</v>
+        <v>Wren Rasmussene</v>
       </c>
       <c r="B145" t="str">
-        <v>leonie.ibarrae37@example.net</v>
+        <v>wren.rasmussene37@example.net</v>
       </c>
       <c r="C145" t="str">
         <v>Yes</v>
@@ -4013,10 +4010,10 @@
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>Alma Prescotte</v>
+        <v>Desmond Sorensene</v>
       </c>
       <c r="B146" t="str">
-        <v>alma.prescotte38@example.net</v>
+        <v>desmond.sorensene38@example.net</v>
       </c>
       <c r="C146" t="str">
         <v>Yes</v>
@@ -4030,10 +4027,10 @@
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>Jonah Whitlocke</v>
+        <v>Rosalind Thackeraye</v>
       </c>
       <c r="B147" t="str">
-        <v>jonah.whitlocke39@example.net</v>
+        <v>rosalind.thackeraye39@example.net</v>
       </c>
       <c r="C147" t="str">
         <v>Yes</v>
@@ -4047,10 +4044,10 @@
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>Beatrice Garnere</v>
+        <v>Caspian Underhille</v>
       </c>
       <c r="B148" t="str">
-        <v>beatrice.garnere40@example.net</v>
+        <v>caspian.underhille40@example.net</v>
       </c>
       <c r="C148" t="str">
         <v>Yes</v>
@@ -4064,10 +4061,10 @@
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>Marcus Nakamurae</v>
+        <v>Odette Valdiviae</v>
       </c>
       <c r="B149" t="str">
-        <v>marcus.nakamurae41@example.net</v>
+        <v>odette.valdiviae41@example.net</v>
       </c>
       <c r="C149" t="str">
         <v>Yes</v>
@@ -4081,10 +4078,10 @@
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>Tamsin Underhille</v>
+        <v>Barnaby Whitlocke</v>
       </c>
       <c r="B150" t="str">
-        <v>tamsin.underhille42@example.net</v>
+        <v>barnaby.whitlocke42@example.net</v>
       </c>
       <c r="C150" t="str">
         <v>Yes</v>
@@ -4098,10 +4095,10 @@
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v>Desmond Ellisone</v>
+        <v>Leonie Arnolde</v>
       </c>
       <c r="B151" t="str">
-        <v>desmond.ellisone43@example.net</v>
+        <v>leonie.arnolde43@example.net</v>
       </c>
       <c r="C151" t="str">
         <v>Yes</v>
@@ -4115,10 +4112,10 @@
     </row>
     <row r="152">
       <c r="A152" t="str">
-        <v>Odette Langforde</v>
+        <v>Tobias Bennette</v>
       </c>
       <c r="B152" t="str">
-        <v>odette.langforde44@example.net</v>
+        <v>tobias.bennette44@example.net</v>
       </c>
       <c r="C152" t="str">
         <v>Yes</v>
@@ -4132,10 +4129,10 @@
     </row>
     <row r="153">
       <c r="A153" t="str">
-        <v>Tobias Sorensene</v>
+        <v>Marisol Castilloe</v>
       </c>
       <c r="B153" t="str">
-        <v>tobias.sorensene45@example.net</v>
+        <v>marisol.castilloe45@example.net</v>
       </c>
       <c r="C153" t="str">
         <v>Yes</v>
@@ -4149,10 +4146,10 @@
     </row>
     <row r="154">
       <c r="A154" t="str">
-        <v>Theo Castilloe</v>
+        <v>Alma Garnere</v>
       </c>
       <c r="B154" t="str">
-        <v>theo.castilloe46@example.net</v>
+        <v>alma.garnere46@example.net</v>
       </c>
       <c r="C154" t="str">
         <v>Yes</v>
@@ -4166,10 +4163,10 @@
     </row>
     <row r="155">
       <c r="A155" t="str">
-        <v>Lucinda Jenningse</v>
+        <v>Theo Hollowaye</v>
       </c>
       <c r="B155" t="str">
-        <v>lucinda.jenningse47@example.net</v>
+        <v>theo.hollowaye47@example.net</v>
       </c>
       <c r="C155" t="str">
         <v>Yes</v>
@@ -4183,10 +4180,10 @@
     </row>
     <row r="156">
       <c r="A156" t="str">
-        <v>Felix Quinteroe</v>
+        <v>Priya Ibarrae</v>
       </c>
       <c r="B156" t="str">
-        <v>felix.quinteroe48@example.net</v>
+        <v>priya.ibarrae48@example.net</v>
       </c>
       <c r="C156" t="str">
         <v>Yes</v>
@@ -4200,10 +4197,10 @@
     </row>
     <row r="157">
       <c r="A157" t="str">
-        <v>Ines Arnolde</v>
+        <v>Jonah Jenningse</v>
       </c>
       <c r="B157" t="str">
-        <v>ines.arnolde49@example.net</v>
+        <v>jonah.jenningse49@example.net</v>
       </c>
       <c r="C157" t="str">
         <v>Yes</v>
@@ -4217,10 +4214,10 @@
     </row>
     <row r="158">
       <c r="A158" t="str">
-        <v>Elliot Hollowaye</v>
+        <v>Lucinda Kowalskie</v>
       </c>
       <c r="B158" t="str">
-        <v>elliot.hollowaye50@example.net</v>
+        <v>lucinda.kowalskie50@example.net</v>
       </c>
       <c r="C158" t="str">
         <v>Yes</v>
@@ -4234,10 +4231,10 @@
     </row>
     <row r="159">
       <c r="A159" t="str">
-        <v>Rosalind Okafore</v>
+        <v>Omar Langforde</v>
       </c>
       <c r="B159" t="str">
-        <v>rosalind.okafore51@example.net</v>
+        <v>omar.langforde51@example.net</v>
       </c>
       <c r="C159" t="str">
         <v>Yes</v>
@@ -4251,10 +4248,10 @@
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v>Barnaby Valdiviae</v>
+        <v>Beatrice Mercere</v>
       </c>
       <c r="B160" t="str">
-        <v>barnaby.valdiviae52@example.net</v>
+        <v>beatrice.mercere52@example.net</v>
       </c>
       <c r="C160" t="str">
         <v>Yes</v>
@@ -4268,10 +4265,10 @@
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>Marisol Fairbankse</v>
+        <v>Felix Nakamurae</v>
       </c>
       <c r="B161" t="str">
-        <v>marisol.fairbankse53@example.net</v>
+        <v>felix.nakamurae53@example.net</v>
       </c>
       <c r="C161" t="str">
         <v>Yes</v>
@@ -4285,10 +4282,10 @@
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>Priya Mercere</v>
+        <v>Harriet Okafore</v>
       </c>
       <c r="B162" t="str">
-        <v>priya.mercere54@example.net</v>
+        <v>harriet.okafore54@example.net</v>
       </c>
       <c r="C162" t="str">
         <v>Yes</v>
@@ -4302,10 +4299,10 @@
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>Omar Thackeraye</v>
+        <v>Marcus Prescotte</v>
       </c>
       <c r="B163" t="str">
-        <v>omar.thackeraye55@example.net</v>
+        <v>marcus.prescotte55@example.net</v>
       </c>
       <c r="C163" t="str">
         <v>Yes</v>
@@ -4319,10 +4316,10 @@
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v>Harriet Dawsone</v>
+        <v>Ines Quinteroe</v>
       </c>
       <c r="B164" t="str">
-        <v>harriet.dawsone56@example.net</v>
+        <v>ines.quinteroe56@example.net</v>
       </c>
       <c r="C164" t="str">
         <v>Yes</v>
@@ -4336,10 +4333,10 @@
     </row>
     <row r="165">
       <c r="A165" t="str">
-        <v>Gordon Kowalskie</v>
+        <v>Gordon Rasmussene</v>
       </c>
       <c r="B165" t="str">
-        <v>gordon.kowalskie57@example.net</v>
+        <v>gordon.rasmussene57@example.net</v>
       </c>
       <c r="C165" t="str">
         <v>Yes</v>
@@ -4353,10 +4350,10 @@
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v>Wren Rasmussene</v>
+        <v>Tamsin Sorensene</v>
       </c>
       <c r="B166" t="str">
-        <v>wren.rasmussene58@example.net</v>
+        <v>tamsin.sorensene58@example.net</v>
       </c>
       <c r="C166" t="str">
         <v>Yes</v>
@@ -4370,10 +4367,10 @@
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>Caspian Bennette</v>
+        <v>Elliot Thackeraye</v>
       </c>
       <c r="B167" t="str">
-        <v>caspian.bennette59@example.net</v>
+        <v>elliot.thackeraye59@example.net</v>
       </c>
       <c r="C167" t="str">
         <v>Yes</v>

</xml_diff>